<commit_message>
chore(content): record Home Credit CTA verification blocker
</commit_message>
<xml_diff>
--- a/docs/content/1phutdangky_Home_Credit_Evergreen_Content_Engine.xlsx
+++ b/docs/content/1phutdangky_Home_Credit_Evergreen_Content_Engine.xlsx
@@ -5278,18 +5278,24 @@
       <x:c r="K5" s="22" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="L5" s="22" t="str">
-        <x:v>Ready</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L5" s="22" t="str">
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M5" s="22" t="str">
         <x:v>Initial 60-day backlog / Day 1</x:v>
       </x:c>
-      <x:c r="N5" s="22"/>
-      <x:c r="O5" s="22"/>
-      <x:c r="P5" s="22"/>
-      <x:c r="Q5" s="22"/>
-      <x:c r="R5" s="22" t="str">
-        <x:v>Core existing money page</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="N5" s="22" t="str">
+        <x:v>2026-10-28</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O5" s="22" t="str">
+        <x:v>https://1phutdangky.com/vay-tien-mat/vay-tien-mat-home-credit-online/</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P5" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q5" s="22" t="str">
+        <x:v>Not requested: content publication blocked</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="R5" s="22" t="str">
+        <x:v>Approved app URL returns HTTP 404 for desktop/iPhone/Android HTTP requests, with and without saCode. AASA/assetlinks are available, but app/store handoff is not verified on a physical device. Keep approved URL and code unchanged. Resume L-PILLAR after verification; do not replace or disable the offer automatically.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -10603,61 +10609,61 @@
       <x:c r="A5" t="str">
         <x:v>Next Queue #</x:v>
       </x:c>
-      <x:c r="B5" t="n">
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B5" t="n">
         <x:f>IFERROR(MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)+4,"DISCOVERY")</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
         <x:v>Next Asset ID</x:v>
       </x:c>
-      <x:c r="B6" t="str">
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B6" t="str">
         <x:f>IF(B5="DISCOVERY","DISCOVERY",INDEX('Evergreen Queue'!$B$5:$B$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
-        <x:v>L-PILLAR</x:v>
+        <x:v>C-PILLAR</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
         <x:v>Topic / Task</x:v>
       </x:c>
-      <x:c r="B7" t="str">
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B7" t="str">
         <x:f>IF(B5="DISCOVERY","Run Discovery Mode",INDEX('Evergreen Queue'!$C$5:$C$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
-        <x:v>Update: Vay tiền mặt Home Credit online</x:v>
+        <x:v>Publish: Mở thẻ tín dụng Home Credit online</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
         <x:v>Product</x:v>
       </x:c>
-      <x:c r="B8" t="str">
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B8" t="str">
         <x:f>IF(B5="DISCOVERY","All",INDEX('Evergreen Queue'!$D$5:$D$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
-        <x:v>Cash Loan</x:v>
+        <x:v>Credit Card</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
         <x:v>Work mode</x:v>
       </x:c>
-      <x:c r="B9" t="str">
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B9" t="str">
         <x:f>IF(B5="DISCOVERY","Research",INDEX('Evergreen Queue'!$F$5:$F$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
-        <x:v>Update existing</x:v>
+        <x:v>New article</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
         <x:v>Canonical / Parent</x:v>
       </x:c>
-      <x:c r="B10" t="str">
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B10" t="str">
         <x:f>IF(B5="DISCOVERY","Evergreen Queue",INDEX('Evergreen Queue'!$H$5:$H$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
-        <x:v>Pillar L</x:v>
+        <x:v>Pillar C</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="B11" t="str">
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B11" t="str">
         <x:f>IF(B5="DISCOVERY","P0",INDEX('Evergreen Queue'!$K$5:$K$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
         <x:v>P0</x:v>
       </x:c>
@@ -10857,22 +10863,54 @@
       <x:c r="A4" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B4" s="22"/>
-      <x:c r="C4" s="22"/>
-      <x:c r="D4" s="22"/>
-      <x:c r="E4" s="22"/>
-      <x:c r="F4" s="22"/>
-      <x:c r="G4" s="22"/>
-      <x:c r="H4" s="22"/>
-      <x:c r="I4" s="22"/>
-      <x:c r="J4" s="22"/>
-      <x:c r="K4" s="22"/>
-      <x:c r="L4" s="22"/>
-      <x:c r="M4" s="22"/>
-      <x:c r="N4" s="22"/>
-      <x:c r="O4" s="22"/>
-      <x:c r="P4" s="22"/>
-      <x:c r="Q4" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B4" s="22" t="str">
+        <x:v>2026-10-28</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C4" s="22" t="str">
+        <x:v>2026-10-28</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D4" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="E4" s="22" t="str">
+        <x:v>L-PILLAR</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="F4" s="22" t="str">
+        <x:v>Update: Vay tiền mặt Home Credit online</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="G4" s="22" t="str">
+        <x:v>Update existing. Preserve canonical URL, UI and approved app referral.</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="H4" s="22" t="str">
+        <x:v>https://1phutdangky.com/vay-tien-mat/vay-tien-mat-home-credit-online/</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="I4" s="22" t="str">
+        <x:v>2026-10-28: https://dangky.homecredit.vn/vay-tien; https://www.homecredit.vn/vay-tien-online-nhanh; https://www.homecredit.vn/faq/vay-tien-mat; https://www.homecredit.vn/blog/cap-nhat-hop-dong-cho-vay-tien-mat; https://www.homecredit.vn/blog/huong-dan-dang-ky-vay-qua-ung-dung-clx-ug; https://www.homecredit.vn/faq/hop-dong-vay; https://www.homecredit.vn/faq/quy-trinh-tham-dinh; https://www.homecredit.vn/lien-he; FAQ-linked loan-rate PDF effective 2026-07-21; approved deeplink; AASA and assetlinks; Apple TN3155 and Android App Links docs.</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="J4" s="22" t="str">
+        <x:v>docs/content/1phutdangky_Home_Credit_Evergreen_Content_Engine.xlsx only</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="K4" s="22" t="str">
+        <x:v>Canonical/update decision passed. Product/source research completed. CTA gate BLOCKED: GET and HEAD 404, iPhone/Android user agents GET 404; /home without query 404; association endpoints 200. No app/store redirect observed. Device-level handoff untested. npm run check PASS: 20 HTML, 18 sitemap URLs; build, Pagefind and validator. No standalone lint/typecheck/test scripts. Workbook recalculation, scope/native-feature checks and git diff --check performed before state commit.</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L4" s="22" t="str">
+        <x:v>No content commit: blocked before implementation</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="M4" s="22" t="str">
+        <x:v>No content push: blocked before implementation; workbook state saved through normal Git workflow</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="N4" s="22" t="str">
+        <x:v>No manual deploy or configuration changes; existing automatic workflow preserved</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O4" s="22" t="str">
+        <x:v>Not performed: no content release</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P4" s="22" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q4" s="22" t="str">
+        <x:v>Required to resume: verify the exact approved URL on a real device with/without the app, or obtain an owner-approved replacement that preserves support-code attribution. Do not infer installed-app failure from HTTP 404. No source-backed article draft or product data changes published. Next selector advances to C-PILLAR, but this invocation stops after this one run.</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="22" t="n">

</xml_diff>

<commit_message>
fix(home-credit): replace app link and refresh loan guide
</commit_message>
<xml_diff>
--- a/docs/content/1phutdangky_Home_Credit_Evergreen_Content_Engine.xlsx
+++ b/docs/content/1phutdangky_Home_Credit_Evergreen_Content_Engine.xlsx
@@ -5279,7 +5279,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L5" s="22" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="M5" s="22" t="str">
         <x:v>Initial 60-day backlog / Day 1</x:v>
@@ -5292,10 +5292,10 @@
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P5" s="22"/>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q5" s="22" t="str">
-        <x:v>Not requested: content publication blocked</x:v>
+        <x:v>Pending GitHub push and automatic Cloudflare deployment</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="R5" s="22" t="str">
-        <x:v>Approved app URL returns HTTP 404 for desktop/iPhone/Android HTTP requests, with and without saCode. AASA/assetlinks are available, but app/store handoff is not verified on a physical device. Keep approved URL and code unchanged. Resume L-PILLAR after verification; do not replace or disable the offer automatically.</x:v>
+        <x:v>Resumed by explicit owner request. Approved public app link replaces broken URL; code 00064470 entered in app. Existing canonical, UI, title ending online and consent-aware analytics preserved.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -10916,22 +10916,52 @@
       <x:c r="A5" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B5" s="22"/>
-      <x:c r="C5" s="22"/>
-      <x:c r="D5" s="22"/>
-      <x:c r="E5" s="22"/>
-      <x:c r="F5" s="22"/>
-      <x:c r="G5" s="22"/>
-      <x:c r="H5" s="22"/>
-      <x:c r="I5" s="22"/>
-      <x:c r="J5" s="22"/>
-      <x:c r="K5" s="22"/>
-      <x:c r="L5" s="22"/>
-      <x:c r="M5" s="22"/>
-      <x:c r="N5" s="22"/>
-      <x:c r="O5" s="22"/>
-      <x:c r="P5" s="22"/>
-      <x:c r="Q5" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B5" s="22" t="str">
+        <x:v>2026-10-28</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C5" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D5" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="E5" s="22" t="str">
+        <x:v>L-PILLAR</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="F5" s="22" t="str">
+        <x:v>Update: Vay tiền mặt Home Credit online</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="G5" s="22" t="str">
+        <x:v>Resume blocked L-PILLAR at owner request; keep URL and UI. Replace app link throughout runtime product/article and complete brief.</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="H5" s="22" t="str">
+        <x:v>https://1phutdangky.com/vay-tien-mat/vay-tien-mat-home-credit-online/</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="I5" s="22" t="str">
+        <x:v>S1/S2/S3/S4/S5 checked 2026-10-28; official app page https://www.homecredit.vn/ung-dung-home-credit; app-flow guide; FAQ-linked loan-rate PDF effective 2026-07-21; contact page. All nine article sources HTTP 200. Published OneLink https://hcv.onelink.me/ausQ/n7wk7jg0: iOS store redirect and Android package vn.homecredit.capp. Owner confirmed link works and app always has support-code field.</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="J5" s="22" t="str">
+        <x:v>src/content/articles/vay-tien-mat/vay-tien-mat-home-credit-online.mdx; src/data/products/loans/home-credit-cash-loan.json; src/components/commercial/ProductCard.astro; docs/content/1phutdangky_Home_Credit_Evergreen_Content_Engine.xlsx</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="K5" s="22" t="str">
+        <x:v>PASS npm run check: build, Pagefind, validator (20 HTML, 18 sitemap URLs). PASS git diff --check. Local Chrome QA: 375/390/768/1440, light/dark, canonical/indexability/JSON-LD, three CTAs, referral-code clipboard, consent denied/granted event gating, no horizontal overflow or page errors. No standalone lint/typecheck/test scripts. Workbook selector recalculated and native features preserved.</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L5" s="22" t="str">
+        <x:v>Pending content commit</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="M5" s="22" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="N5" s="22" t="str">
+        <x:v>Existing GitHub-to-Cloudflare workflow; awaiting production</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O5" s="22" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P5" s="22" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q5" s="22" t="str">
+        <x:v>Resume run 1 as run 2, not C-PILLAR. Keep original blocked history. Retain owner-approved short title and add no links to unpublished support/card routes. One content cycle only.</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="22" t="n">
@@ -19531,8 +19561,8 @@
       <x:c r="C5" s="22" t="str">
         <x:v>SEO Title</x:v>
       </x:c>
-      <x:c r="D5" s="22" t="str">
-        <x:v>Vay tiền mặt Home Credit online: Điều kiện, lãi suất và cách đăng ký</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D5" s="22" t="str">
+        <x:v>Hướng dẫn vay tiền mặt Home Credit online</x:v>
       </x:c>
       <x:c r="E5" s="22" t="str">
         <x:v>Transactional loan</x:v>
@@ -19570,8 +19600,8 @@
       <x:c r="P5" s="22" t="str">
         <x:v>Keep existing URL</x:v>
       </x:c>
-      <x:c r="Q5" s="22" t="str">
-        <x:v>Giữ URL hiện tại.</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q5" s="22" t="str">
+        <x:v>Giữ URL và tiêu đề đã được chủ website chốt, có online ở cuối.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -19584,8 +19614,8 @@
       <x:c r="C6" s="22" t="str">
         <x:v>H1</x:v>
       </x:c>
-      <x:c r="D6" s="22" t="str">
-        <x:v>Vay tiền mặt Home Credit online: Cách đăng ký, chi phí và điều cần kiểm tra</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D6" s="22" t="str">
+        <x:v>Hướng dẫn vay tiền mặt Home Credit online</x:v>
       </x:c>
       <x:c r="E6" s="22" t="str">
         <x:v>Transactional + decision</x:v>
@@ -19823,8 +19853,8 @@
       <x:c r="L10" s="22" t="str">
         <x:v>L-REJECT</x:v>
       </x:c>
-      <x:c r="M10" s="22" t="str">
-        <x:v>https://dangky.homecredit.vn/vay-tien</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="M10" s="22" t="str">
+        <x:v>https://www.homecredit.vn/blog/huong-dan-dang-ky-vay-qua-ung-dung-clx-ug</x:v>
       </x:c>
       <x:c r="N10" s="22" t="str">
         <x:v>Current flow</x:v>
@@ -21126,8 +21156,8 @@
       <x:c r="B5" s="22" t="str">
         <x:v>Hot</x:v>
       </x:c>
-      <x:c r="C5" s="22" t="str">
-        <x:v>Kiểm tra/đăng ký khoản vay trên kênh Home Credit qua link</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C5" s="22" t="str">
+        <x:v>Tải ứng dụng Home Credit</x:v>
       </x:c>
       <x:c r="D5" s="22" t="str">
         <x:v>Xem điều kiện và chi phí trước</x:v>
@@ -21147,8 +21177,8 @@
       <x:c r="I5" s="22" t="str">
         <x:v>Không hứa duyệt/hạn mức</x:v>
       </x:c>
-      <x:c r="J5" s="22" t="str">
-        <x:v>cta_hc_loan; outbound_hc_loan</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="J5" s="22" t="str">
+        <x:v>affiliate_click; referral_code_copy (existing consent-aware events)</x:v>
       </x:c>
       <x:c r="K5" s="22" t="str">
         <x:v>Outbound CTR / approved conversion if available</x:v>
@@ -21815,8 +21845,8 @@
       <x:c r="H5" s="22" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="I5" s="22" t="str">
-        <x:v>2026-10-27</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="I5" s="22" t="str">
+        <x:v>2026-10-28</x:v>
       </x:c>
       <x:c r="J5" s="22" t="str">
         <x:v>Before publish/update</x:v>
@@ -21853,8 +21883,8 @@
       <x:c r="H6" s="22" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="I6" s="22" t="str">
-        <x:v>2026-10-27</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="I6" s="22" t="str">
+        <x:v>2026-10-28</x:v>
       </x:c>
       <x:c r="J6" s="22" t="str">
         <x:v>Before cost update</x:v>
@@ -21891,8 +21921,8 @@
       <x:c r="H7" s="22" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="I7" s="22" t="str">
-        <x:v>2026-10-27</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="I7" s="22" t="str">
+        <x:v>2026-10-28</x:v>
       </x:c>
       <x:c r="J7" s="22" t="str">
         <x:v>Before eligibility update</x:v>
@@ -21929,8 +21959,8 @@
       <x:c r="H8" s="22" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="I8" s="22" t="str">
-        <x:v>2026-10-27</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="I8" s="22" t="str">
+        <x:v>2026-10-28</x:v>
       </x:c>
       <x:c r="J8" s="22" t="str">
         <x:v>Before troubleshooting publish</x:v>
@@ -21967,8 +21997,8 @@
       <x:c r="H9" s="22" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="I9" s="22" t="str">
-        <x:v>2026-10-27</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="I9" s="22" t="str">
+        <x:v>2026-10-28</x:v>
       </x:c>
       <x:c r="J9" s="22" t="str">
         <x:v>Before publish</x:v>
@@ -22157,8 +22187,8 @@
       <x:c r="H14" s="22" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="I14" s="22" t="str">
-        <x:v>2026-10-27</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="I14" s="22" t="str">
+        <x:v>2026-10-28</x:v>
       </x:c>
       <x:c r="J14" s="22" t="str">
         <x:v>Before Codex batch</x:v>

</xml_diff>

<commit_message>
chore(content): record Home Credit production verification
</commit_message>
<xml_diff>
--- a/docs/content/1phutdangky_Home_Credit_Evergreen_Content_Engine.xlsx
+++ b/docs/content/1phutdangky_Home_Credit_Evergreen_Content_Engine.xlsx
@@ -5279,7 +5279,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L5" s="22" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M5" s="22" t="str">
         <x:v>Initial 60-day backlog / Day 1</x:v>
@@ -5290,9 +5290,11 @@
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O5" s="22" t="str">
         <x:v>https://1phutdangky.com/vay-tien-mat/vay-tien-mat-home-credit-online/</x:v>
       </x:c>
-      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P5" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P5" s="22" t="str">
+        <x:v>50f56521c5afae1afc102cbc694d1fd6b68619b2</x:v>
+      </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q5" s="22" t="str">
-        <x:v>Pending GitHub push and automatic Cloudflare deployment</x:v>
+        <x:v>Cloudflare Pages success fcfa3d65-3191-4ac5-8d28-8498798a6986; production verified 2026-10-28</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="R5" s="22" t="str">
         <x:v>Resumed by explicit owner request. Approved public app link replaces broken URL; code 00064470 entered in app. Existing canonical, UI, title ending online and consent-aware analytics preserved.</x:v>
@@ -10919,7 +10921,9 @@
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B5" s="22" t="str">
         <x:v>2026-10-28</x:v>
       </x:c>
-      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C5" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C5" s="22" t="str">
+        <x:v>2026-10-28</x:v>
+      </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D5" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -10945,19 +10949,19 @@
         <x:v>PASS npm run check: build, Pagefind, validator (20 HTML, 18 sitemap URLs). PASS git diff --check. Local Chrome QA: 375/390/768/1440, light/dark, canonical/indexability/JSON-LD, three CTAs, referral-code clipboard, consent denied/granted event gating, no horizontal overflow or page errors. No standalone lint/typecheck/test scripts. Workbook selector recalculated and native features preserved.</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L5" s="22" t="str">
-        <x:v>Pending content commit</x:v>
+        <x:v>50f56521c5afae1afc102cbc694d1fd6b68619b2</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="M5" s="22" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Content commit pushed to origin/main; GitHub SHA verified</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="N5" s="22" t="str">
-        <x:v>Existing GitHub-to-Cloudflare workflow; awaiting production</x:v>
+        <x:v>Cloudflare Pages check SUCCESS; deployment fcfa3d65-3191-4ac5-8d28-8498798a6986 via existing Git integration</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O5" s="22" t="str">
-        <x:v>Pending</x:v>
+        <x:v>PASS production HTTP 200; 3 exact OneLink CTAs, support code, canonical, title/meta/schema/sitemap; responsive light/dark and consent-aware event/copy checks repeated</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P5" s="22" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q5" s="22" t="str">
         <x:v>Resume run 1 as run 2, not C-PILLAR. Keep original blocked history. Retain owner-approved short title and add no links to unpublished support/card routes. One content cycle only.</x:v>

</xml_diff>

<commit_message>
feat(content): publish Home Credit credit card guide
</commit_message>
<xml_diff>
--- a/docs/content/1phutdangky_Home_Credit_Evergreen_Content_Engine.xlsx
+++ b/docs/content/1phutdangky_Home_Credit_Evergreen_Content_Engine.xlsx
@@ -5334,18 +5334,24 @@
       <x:c r="K6" s="22" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="L6" s="22" t="str">
-        <x:v>Ready</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L6" s="22" t="str">
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="M6" s="22" t="str">
         <x:v>Initial 60-day backlog / Day 2</x:v>
       </x:c>
-      <x:c r="N6" s="22"/>
-      <x:c r="O6" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="N6" s="22" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O6" s="22" t="str">
+        <x:v>https://1phutdangky.com/the-tin-dung/mo-the-tin-dung-home-credit-online/</x:v>
+      </x:c>
       <x:c r="P6" s="22"/>
-      <x:c r="Q6" s="22"/>
-      <x:c r="R6" s="22" t="str">
-        <x:v>Second money page</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q6" s="22" t="str">
+        <x:v>Pending push and existing Cloudflare deployment</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="R6" s="22" t="str">
+        <x:v>Queue2 C-PILLAR only. New separate credit-card product and pillar; exact owner-approved generic App OneLink and support code00064470, no card-specific attribution/approval promise. Current04Sep2026 tariff columns and16Jul2026 TnC govern; distinct loan owner retained with reciprocal bridge. Shared UI/title visuals untouched.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -10612,8 +10618,8 @@
         <x:v>Next Queue #</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B5" t="n">
-        <x:f>IFERROR(MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)+4,"DISCOVERY")</x:f>
-        <x:v>6</x:v>
+        <x:f>IFERROR(INDEX('Evergreen Queue'!$A$5:$A$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)),"DISCOVERY")</x:f>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -10622,7 +10628,7 @@
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B6" t="str">
         <x:f>IF(B5="DISCOVERY","DISCOVERY",INDEX('Evergreen Queue'!$B$5:$B$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
-        <x:v>C-PILLAR</x:v>
+        <x:v>L-RATE</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -10631,7 +10637,7 @@
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B7" t="str">
         <x:f>IF(B5="DISCOVERY","Run Discovery Mode",INDEX('Evergreen Queue'!$C$5:$C$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
-        <x:v>Publish: Mở thẻ tín dụng Home Credit online</x:v>
+        <x:v>Lãi suất vay tiền mặt Home Credit: cách đọc</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -10640,7 +10646,7 @@
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B8" t="str">
         <x:f>IF(B5="DISCOVERY","All",INDEX('Evergreen Queue'!$D$5:$D$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
-        <x:v>Credit Card</x:v>
+        <x:v>Cash Loan</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -10658,7 +10664,7 @@
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B10" t="str">
         <x:f>IF(B5="DISCOVERY","Evergreen Queue",INDEX('Evergreen Queue'!$H$5:$H$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
-        <x:v>Pillar C</x:v>
+        <x:v>Pillar L</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -10971,22 +10977,52 @@
       <x:c r="A6" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B6" s="22"/>
-      <x:c r="C6" s="22"/>
-      <x:c r="D6" s="22"/>
-      <x:c r="E6" s="22"/>
-      <x:c r="F6" s="22"/>
-      <x:c r="G6" s="22"/>
-      <x:c r="H6" s="22"/>
-      <x:c r="I6" s="22"/>
-      <x:c r="J6" s="22"/>
-      <x:c r="K6" s="22"/>
-      <x:c r="L6" s="22"/>
-      <x:c r="M6" s="22"/>
-      <x:c r="N6" s="22"/>
-      <x:c r="O6" s="22"/>
-      <x:c r="P6" s="22"/>
-      <x:c r="Q6" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B6" s="22" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C6" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D6" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="E6" s="22" t="str">
+        <x:v>C-PILLAR</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="F6" s="22" t="str">
+        <x:v>Publish: Mở thẻ tín dụng Home Credit online</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="G6" s="22" t="str">
+        <x:v>New standalone card owner; first eligible Ready (actual Queue2, worksheet row6). Cash-loan owner retained. Verify S6/S7/S8 and approved app CTA before implementation.</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="H6" s="22" t="str">
+        <x:v>https://1phutdangky.com/the-tin-dung/mo-the-tin-dung-home-credit-online/</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="I6" s="22" t="str">
+        <x:v>2026-10-29 S6 official cardpage(updated12Oct2026), S7 cardFAQ, S8 contractlookup: latest linked tariff04Sep2026, cardTnC16Jul2026 and installmentTnC04Sep2026. Tariff2pages visually checked:4cardtypes, standard39k managementfee exception3M/5tx,49.5%annualinterest; onlinecard noATM, minimum formula includes installment/pastdue, latefee0.12%/day min150k/max1M collection5/35/65days. CardTnC5.1/5.2/5.4 for grace/fullpayment, cashinterestfromposting and unpaid-minimumlatefee. All7articlesourceURLsHTTP200. Approved generic OneLink iPhone301 to itms-appss AppStoreid1553761073; Android200app/storedispatcher. Nativeinstalled-app handoff and card attribution not claimed. Owner-supplied appstaffcodefield/code preserved.</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="J6" s="22" t="str">
+        <x:v>src/content/articles/the-tin-dung/mo-the-tin-dung-home-credit-online.mdx; src/data/products/credit-cards/home-credit-credit-card.json; src/content/articles/vay-tien-mat/vay-tien-mat-home-credit-online.mdx; docs/content/1phutdangky_Home_Credit_Evergreen_Content_Engine.xlsx. Social images generated by existing build endpoint; no separate cover.</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="K6" s="22" t="str">
+        <x:v>PASS npm run check: Astro build/Pagefind/validator24HTML/22sitemapURLs. PASS git diff --check. LocalChrome375/390/768/1440 light/dark: oneH1, title/card/OG/Twitter sync, canonical/Article/BreadcrumbList, TOC anchors, sitemaponce, Pagefind, homepage/category and reciprocal loanlinks. Three exact AppCTAs;00064470clipboard; correct separate cardproduct/eventidentity; consentdenied/granted affiliate_click/referral_code_copy. Existingloan3CTA destinations/title retained; nooverflow/runtimeerrors. Independenteditorial/source review; corrected ambiguouslatefee trigger. No separate lint/typecheck/testscripts. Workbookrecalculation and nativefeaturepreservation checked.</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L6" s="22" t="str">
+        <x:v>Pending content commit</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="M6" s="22" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="N6" s="22" t="str">
+        <x:v>Existing automatic GitHub/Cloudflare Pages integration</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O6" s="22" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P6" s="22" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q6" s="22" t="str">
+        <x:v>New card owner; loan productJSON unchanged and loanarticle only reciprocal link/update date. Title ends online. Generic AppCTA not a card-specific deeplink; staffcode not labelled cardreferralcode. Shared UI/analytics/deploymentconfig unchanged. Fixed NextAction B5: old formula returned Excelrow6 as Queue#; changed only this formula to INDEX actualqueueID (nootherformula depends on its numeric row). Refreshed selector correctly points Queue3 L-RATE. Prior blocked/resume history preserved.</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="22" t="n">
@@ -19936,8 +19972,8 @@
       <x:c r="C12" s="22" t="str">
         <x:v>SEO Title</x:v>
       </x:c>
-      <x:c r="D12" s="22" t="str">
-        <x:v>Mở thẻ tín dụng Home Credit online: Điều kiện, phí và cách đăng ký</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D12" s="22" t="str">
+        <x:v>Hướng dẫn mở thẻ tín dụng Home Credit online</x:v>
       </x:c>
       <x:c r="E12" s="22" t="str">
         <x:v>Transactional card</x:v>
@@ -19975,8 +20011,8 @@
       <x:c r="P12" s="22" t="str">
         <x:v>Publish</x:v>
       </x:c>
-      <x:c r="Q12" s="22" t="str">
-        <x:v>Second money page.</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q12" s="22" t="str">
+        <x:v>Published title-only shared visual. Separate card product; approved generic App OneLink and app-level staffcode00064470; no card-attribution or approval guarantee. Current tariff04Sep2026 and TnC16Jul2026; scope card owner distinct from cash loan.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -19989,8 +20025,8 @@
       <x:c r="C13" s="22" t="str">
         <x:v>H1</x:v>
       </x:c>
-      <x:c r="D13" s="22" t="str">
-        <x:v>Mở thẻ tín dụng Home Credit online: Điều kiện, hạn mức, phí và cách dùng</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D13" s="22" t="str">
+        <x:v>Hướng dẫn mở thẻ tín dụng Home Credit online</x:v>
       </x:c>
       <x:c r="E13" s="22" t="str">
         <x:v>Transactional + decision</x:v>
@@ -20042,8 +20078,8 @@
       <x:c r="C14" s="22" t="str">
         <x:v>Answer block</x:v>
       </x:c>
-      <x:c r="D14" s="22" t="str">
-        <x:v>Thẻ tín dụng Home Credit có thể được đăng ký online; Home Credit thẩm định hồ sơ và quyết định cấp thẻ/hạn mức. Trước khi đăng ký, cần kiểm biểu phí, lãi suất, ngày sao kê và số tiền tối thiểu phải thanh toán theo điều khoản hiện hành.</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D14" s="22" t="str">
+        <x:v>Bạn có thể đăng ký thẻ tín dụng qua ứng dụng Home Credit. Home Credit thẩm định hồ sơ và quyết định cấp thẻ, hạn mức. Trước khi ký, kiểm tra đúng loại thẻ, phí quản lý, lãi suất và nghĩa vụ thanh toán; miễn phí thường niên không có nghĩa mọi chi phí sử dụng đều bằng 0.</x:v>
       </x:c>
       <x:c r="E14" s="22" t="str">
         <x:v>Card intent</x:v>
@@ -21201,11 +21237,11 @@
       <x:c r="B6" s="22" t="str">
         <x:v>Hot</x:v>
       </x:c>
-      <x:c r="C6" s="22" t="str">
-        <x:v>Mở thẻ tín dụng Home Credit</x:v>
-      </x:c>
-      <x:c r="D6" s="22" t="str">
-        <x:v>Xem phí/lãi trước khi đăng ký</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C6" s="22" t="str">
+        <x:v>Tải ứng dụng Home Credit</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D6" s="22" t="str">
+        <x:v>Mục lục: Phí và lãi cần đọc trước khi ký</x:v>
       </x:c>
       <x:c r="E6" s="22" t="str">
         <x:v>High</x:v>
@@ -21222,8 +21258,8 @@
       <x:c r="I6" s="22" t="str">
         <x:v>Không hứa hạn mức/approval</x:v>
       </x:c>
-      <x:c r="J6" s="22" t="str">
-        <x:v>cta_hc_card; outbound_hc_card</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="J6" s="22" t="str">
+        <x:v>affiliate_click; referral_code_copy (existing consent-aware events, separate credit-card product ID)</x:v>
       </x:c>
       <x:c r="K6" s="22" t="str">
         <x:v>Outbound CTR / card conversion</x:v>
@@ -22039,8 +22075,8 @@
       <x:c r="H10" s="22" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="I10" s="22" t="str">
-        <x:v>2026-10-27</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="I10" s="22" t="str">
+        <x:v>2026-10-29</x:v>
       </x:c>
       <x:c r="J10" s="22" t="str">
         <x:v>Before card update</x:v>
@@ -22048,8 +22084,8 @@
       <x:c r="K10" s="22" t="str">
         <x:v>Required</x:v>
       </x:c>
-      <x:c r="L10" s="22" t="str">
-        <x:v>Current page states 20–60, valid ID, online opening; verify current product page.</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L10" s="22" t="str">
+        <x:v>2026-10-29 productpage accessed200, pageupdated12Oct2026. Eligibility20-60/validID, range1-100M, Apphome optionUu dai the tin dung. Age paragraph scoped Vietnamese customers; no approval guarantee or card-specific supportcode placement assumed.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -22077,8 +22113,8 @@
       <x:c r="H11" s="22" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="I11" s="22" t="str">
-        <x:v>2026-10-27</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="I11" s="22" t="str">
+        <x:v>2026-10-29</x:v>
       </x:c>
       <x:c r="J11" s="22" t="str">
         <x:v>Before lifecycle update</x:v>
@@ -22086,8 +22122,8 @@
       <x:c r="K11" s="22" t="str">
         <x:v>Required</x:v>
       </x:c>
-      <x:c r="L11" s="22" t="str">
-        <x:v>Useful operational source.</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L11" s="22" t="str">
+        <x:v>2026-10-29 FAQ200. Supports Appapplication, activation and cardhotline1900633999. For minimum payment and fees use latest tariff/TnC instead of simplified7%FAQ or blanketATMavailability for virtualcards.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -22115,8 +22151,8 @@
       <x:c r="H12" s="22" t="str">
         <x:v>Very High</x:v>
       </x:c>
-      <x:c r="I12" s="22" t="str">
-        <x:v>2026-10-27</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="I12" s="22" t="str">
+        <x:v>2026-10-29</x:v>
       </x:c>
       <x:c r="J12" s="22" t="str">
         <x:v>Every publish/update involving fees</x:v>
@@ -22124,8 +22160,8 @@
       <x:c r="K12" s="22" t="str">
         <x:v>Latest document wins</x:v>
       </x:c>
-      <x:c r="L12" s="22" t="str">
-        <x:v>Page currently lists tariff effective 04/09/2026 and installment terms same date.</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L12" s="22" t="str">
+        <x:v>2026-10-29 lookup200: latest tariff04Sep2026/2609_Credit_Card_tariff_VN_ff1e281fb6.pdf; latest cardTnC16Jul2026/Card_Card_Tn_C_VN_ver07_2026_0950fb1dfe.pdf; installmentTnC04Sep2026/Revamped_EPP_Tn_C_04092026_final_3_22e282cae2.pdf. Both tariffpages visually checked; cardtype/date exceptions preserved.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -22147,14 +22183,14 @@
       <x:c r="F13" s="22" t="str">
         <x:v>Loan approval guarantee</x:v>
       </x:c>
-      <x:c r="G13" s="22" t="str">
-        <x:v>L-PAY</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="G13" s="22" t="str">
+        <x:v>C-PILLAR; L-PAY</x:v>
       </x:c>
       <x:c r="H13" s="22" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="I13" s="22" t="str">
-        <x:v>2026-10-27</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="I13" s="22" t="str">
+        <x:v>2026-10-29</x:v>
       </x:c>
       <x:c r="J13" s="22" t="str">
         <x:v>Before servicing update</x:v>

</xml_diff>

<commit_message>
chore(content): record Home Credit card production verification
</commit_message>
<xml_diff>
--- a/docs/content/1phutdangky_Home_Credit_Evergreen_Content_Engine.xlsx
+++ b/docs/content/1phutdangky_Home_Credit_Evergreen_Content_Engine.xlsx
@@ -5335,7 +5335,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L6" s="22" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M6" s="22" t="str">
         <x:v>Initial 60-day backlog / Day 2</x:v>
@@ -5346,9 +5346,11 @@
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O6" s="22" t="str">
         <x:v>https://1phutdangky.com/the-tin-dung/mo-the-tin-dung-home-credit-online/</x:v>
       </x:c>
-      <x:c r="P6" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P6" s="22" t="str">
+        <x:v>273e42760718aa80e4c68301cca0c0bab0f2c8ea</x:v>
+      </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q6" s="22" t="str">
-        <x:v>Pending push and existing Cloudflare deployment</x:v>
+        <x:v>Cloudflare Pages success 406a64e3-c6f8-498e-bd9b-e771fb96d869; production verified 2026-10-29</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="R6" s="22" t="str">
         <x:v>Queue2 C-PILLAR only. New separate credit-card product and pillar; exact owner-approved generic App OneLink and support code00064470, no card-specific attribution/approval promise. Current04Sep2026 tariff columns and16Jul2026 TnC govern; distinct loan owner retained with reciprocal bridge. Shared UI/title visuals untouched.</x:v>
@@ -10980,7 +10982,9 @@
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B6" s="22" t="str">
         <x:v>2026-10-29</x:v>
       </x:c>
-      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C6" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C6" s="22" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D6" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -11006,19 +11010,19 @@
         <x:v>PASS npm run check: Astro build/Pagefind/validator24HTML/22sitemapURLs. PASS git diff --check. LocalChrome375/390/768/1440 light/dark: oneH1, title/card/OG/Twitter sync, canonical/Article/BreadcrumbList, TOC anchors, sitemaponce, Pagefind, homepage/category and reciprocal loanlinks. Three exact AppCTAs;00064470clipboard; correct separate cardproduct/eventidentity; consentdenied/granted affiliate_click/referral_code_copy. Existingloan3CTA destinations/title retained; nooverflow/runtimeerrors. Independenteditorial/source review; corrected ambiguouslatefee trigger. No separate lint/typecheck/testscripts. Workbookrecalculation and nativefeaturepreservation checked.</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L6" s="22" t="str">
-        <x:v>Pending content commit</x:v>
+        <x:v>273e42760718aa80e4c68301cca0c0bab0f2c8ea</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="M6" s="22" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Pushed origin/main; remote SHA verified equal to content commit.</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="N6" s="22" t="str">
-        <x:v>Existing automatic GitHub/Cloudflare Pages integration</x:v>
+        <x:v>Existing automatic GitHub/Cloudflare Pages integration: success 406a64e3-c6f8-498e-bd9b-e771fb96d869</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O6" s="22" t="str">
-        <x:v>Pending</x:v>
+        <x:v>PASS 2026-10-29 production Chrome 375/390/768/1440 light/dark: route200, oneH1; synchronized title/card/OG/Twitter/generatedPNG200; canonical/Article/BreadcrumbList; 22sitemapURLs/newrouteonce; Pagefind; homepage/category/reciprocal loanbridge; three exact approved AppCTAs; code00064470copy; correct cardproduct identity; consentdenied/granted events; existingloan title/3CTAs unchanged; no overflow or runtimeerrors. Production390light/1440dark visually reviewed.</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P6" s="22" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q6" s="22" t="str">
         <x:v>New card owner; loan productJSON unchanged and loanarticle only reciprocal link/update date. Title ends online. Generic AppCTA not a card-specific deeplink; staffcode not labelled cardreferralcode. Shared UI/analytics/deploymentconfig unchanged. Fixed NextAction B5: old formula returned Excelrow6 as Queue#; changed only this formula to INDEX actualqueueID (nootherformula depends on its numeric row). Refreshed selector correctly points Queue3 L-RATE. Prior blocked/resume history preserved.</x:v>

</xml_diff>